<commit_message>
auto: reporte semana 2026-07-20 → 2026-07-26
</commit_message>
<xml_diff>
--- a/INFORME EXCESOS DE VELOCIDAD.xlsx
+++ b/INFORME EXCESOS DE VELOCIDAD.xlsx
@@ -874,7 +874,6 @@
           <t>EN_0364 (Lux)</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr"/>
       <c r="C6" t="n">
         <v>1</v>
       </c>
@@ -935,7 +934,6 @@
           <t>EN_0364 (Lux)</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr"/>
       <c r="C7" t="n">
         <v>2</v>
       </c>
@@ -996,7 +994,6 @@
           <t>EN_0364 (Lux)</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr"/>
       <c r="C8" t="n">
         <v>3</v>
       </c>
@@ -1057,7 +1054,6 @@
           <t>EN_0364 (Lux)</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr"/>
       <c r="C9" t="n">
         <v>4</v>
       </c>
@@ -1118,7 +1114,6 @@
           <t>EN_0364 (Lux)</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr"/>
       <c r="C10" t="n">
         <v>5</v>
       </c>
@@ -1179,7 +1174,6 @@
           <t>EN_0364 (Lux)</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr"/>
       <c r="C11" t="n">
         <v>6</v>
       </c>
@@ -1240,7 +1234,6 @@
           <t>EN_0364 (Lux)</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr"/>
       <c r="C12" t="n">
         <v>7</v>
       </c>
@@ -1301,7 +1294,6 @@
           <t>EN_0364 (Lux)</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr"/>
       <c r="C13" t="n">
         <v>8</v>
       </c>
@@ -1362,7 +1354,6 @@
           <t>EN_0364 (Lux)</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr"/>
       <c r="C14" t="n">
         <v>9</v>
       </c>
@@ -1421,7 +1412,6 @@
           <t>EN_0364 (Lux)</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr"/>
       <c r="C15" t="n">
         <v>10</v>
       </c>
@@ -1480,7 +1470,6 @@
           <t>PEUGEOT SVCH-53 (STGO)</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr"/>
       <c r="C16" t="n">
         <v>1</v>
       </c>
@@ -1539,7 +1528,6 @@
           <t>EN_0378 (LUX)</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr"/>
       <c r="C17" t="n">
         <v>1</v>
       </c>
@@ -1600,7 +1588,6 @@
           <t>EN_0378 (LUX)</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr"/>
       <c r="C18" t="n">
         <v>2</v>
       </c>
@@ -1661,7 +1648,6 @@
           <t>EN_0378 (LUX)</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr"/>
       <c r="C19" t="n">
         <v>3</v>
       </c>
@@ -1722,7 +1708,6 @@
           <t>EN_0364 (Lux)</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr"/>
       <c r="C20" t="n">
         <v>11</v>
       </c>
@@ -1783,7 +1768,6 @@
           <t>EN_0364 (Lux)</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr"/>
       <c r="C21" t="n">
         <v>12</v>
       </c>
@@ -1844,7 +1828,6 @@
           <t>EN_0364 (Lux)</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr"/>
       <c r="C22" t="n">
         <v>13</v>
       </c>
@@ -1905,7 +1888,6 @@
           <t>EN_0364 (Lux)</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr"/>
       <c r="C23" t="n">
         <v>14</v>
       </c>
@@ -1966,7 +1948,6 @@
           <t>EN_0364 (Lux)</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr"/>
       <c r="C24" t="n">
         <v>15</v>
       </c>
@@ -2027,7 +2008,6 @@
           <t>EN_0364 (Lux)</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr"/>
       <c r="C25" t="n">
         <v>16</v>
       </c>
@@ -2088,7 +2068,6 @@
           <t>EN_0364 (Lux)</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr"/>
       <c r="C26" t="n">
         <v>17</v>
       </c>
@@ -2149,7 +2128,6 @@
           <t>MAXUS TVVB-25 (CHILLAN)</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr"/>
       <c r="C27" t="n">
         <v>1</v>
       </c>
@@ -2208,7 +2186,6 @@
           <t>MAXUS VGVV-79 (STGO MA)</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr"/>
       <c r="C28" t="n">
         <v>1</v>
       </c>

</xml_diff>

<commit_message>
auto: reporte semana 2026-07-27 → 2026-08-02
</commit_message>
<xml_diff>
--- a/INFORME EXCESOS DE VELOCIDAD.xlsx
+++ b/INFORME EXCESOS DE VELOCIDAD.xlsx
@@ -2213,7 +2213,6 @@
           <t>MAXUS TVVB-25 (CHILLAN)</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr"/>
       <c r="C29" t="n">
         <v>1</v>
       </c>
@@ -2272,7 +2271,6 @@
           <t>MITSUBISHI VDYZ-59 (Copiapo)</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr"/>
       <c r="C30" t="n">
         <v>1</v>
       </c>
@@ -2331,7 +2329,6 @@
           <t>EN_0364 (Lux)</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr"/>
       <c r="C31" t="n">
         <v>1</v>
       </c>
@@ -2392,7 +2389,6 @@
           <t>EN_0364 (Lux)</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr"/>
       <c r="C32" t="n">
         <v>2</v>
       </c>
@@ -2453,7 +2449,6 @@
           <t>EN_0364 (Lux)</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr"/>
       <c r="C33" t="n">
         <v>3</v>
       </c>
@@ -2514,7 +2509,6 @@
           <t>EN_0364 (Lux)</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr"/>
       <c r="C34" t="n">
         <v>4</v>
       </c>
@@ -2575,7 +2569,6 @@
           <t>EN_0364 (Lux)</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr"/>
       <c r="C35" t="n">
         <v>5</v>
       </c>
@@ -2636,7 +2629,6 @@
           <t>EN_0364 (Lux)</t>
         </is>
       </c>
-      <c r="B36" t="inlineStr"/>
       <c r="C36" t="n">
         <v>6</v>
       </c>
@@ -2697,7 +2689,6 @@
           <t>EN_0364 (Lux)</t>
         </is>
       </c>
-      <c r="B37" t="inlineStr"/>
       <c r="C37" t="n">
         <v>7</v>
       </c>
@@ -2758,7 +2749,6 @@
           <t>EN_0364 (Lux)</t>
         </is>
       </c>
-      <c r="B38" t="inlineStr"/>
       <c r="C38" t="n">
         <v>8</v>
       </c>
@@ -2819,7 +2809,6 @@
           <t>EN_0364 (Lux)</t>
         </is>
       </c>
-      <c r="B39" t="inlineStr"/>
       <c r="C39" t="n">
         <v>9</v>
       </c>
@@ -2880,7 +2869,6 @@
           <t>EN_0364 (Lux)</t>
         </is>
       </c>
-      <c r="B40" t="inlineStr"/>
       <c r="C40" t="n">
         <v>10</v>
       </c>
@@ -2941,7 +2929,6 @@
           <t>EN_0364 (Lux)</t>
         </is>
       </c>
-      <c r="B41" t="inlineStr"/>
       <c r="C41" t="n">
         <v>11</v>
       </c>
@@ -3002,7 +2989,6 @@
           <t>EN_0364 (Lux)</t>
         </is>
       </c>
-      <c r="B42" t="inlineStr"/>
       <c r="C42" t="n">
         <v>12</v>
       </c>
@@ -3063,7 +3049,6 @@
           <t>EN_0364 (Lux)</t>
         </is>
       </c>
-      <c r="B43" t="inlineStr"/>
       <c r="C43" t="n">
         <v>13</v>
       </c>
@@ -3124,7 +3109,6 @@
           <t>EN_0364 (Lux)</t>
         </is>
       </c>
-      <c r="B44" t="inlineStr"/>
       <c r="C44" t="n">
         <v>14</v>
       </c>
@@ -3185,7 +3169,6 @@
           <t>EN_0364 (Lux)</t>
         </is>
       </c>
-      <c r="B45" t="inlineStr"/>
       <c r="C45" t="n">
         <v>15</v>
       </c>
@@ -3246,7 +3229,6 @@
           <t>EN_0364 (Lux)</t>
         </is>
       </c>
-      <c r="B46" t="inlineStr"/>
       <c r="C46" t="n">
         <v>16</v>
       </c>
@@ -3307,7 +3289,6 @@
           <t>EN_0364 (Lux)</t>
         </is>
       </c>
-      <c r="B47" t="inlineStr"/>
       <c r="C47" t="n">
         <v>17</v>
       </c>
@@ -3368,7 +3349,6 @@
           <t>EN_0364 (Lux)</t>
         </is>
       </c>
-      <c r="B48" t="inlineStr"/>
       <c r="C48" t="n">
         <v>19</v>
       </c>
@@ -3429,7 +3409,6 @@
           <t>EN_0364 (Lux)</t>
         </is>
       </c>
-      <c r="B49" t="inlineStr"/>
       <c r="C49" t="n">
         <v>20</v>
       </c>
@@ -3490,7 +3469,6 @@
           <t>EN_0364 (Lux)</t>
         </is>
       </c>
-      <c r="B50" t="inlineStr"/>
       <c r="C50" t="n">
         <v>21</v>
       </c>
@@ -3551,7 +3529,6 @@
           <t>EN_0364 (Lux)</t>
         </is>
       </c>
-      <c r="B51" t="inlineStr"/>
       <c r="C51" t="n">
         <v>22</v>
       </c>
@@ -3612,7 +3589,6 @@
           <t>EN_0364 (Lux)</t>
         </is>
       </c>
-      <c r="B52" t="inlineStr"/>
       <c r="C52" t="n">
         <v>23</v>
       </c>
@@ -3673,7 +3649,6 @@
           <t>EN_0364 (Lux)</t>
         </is>
       </c>
-      <c r="B53" t="inlineStr"/>
       <c r="C53" t="n">
         <v>24</v>
       </c>
@@ -3734,7 +3709,6 @@
           <t>EN_0364 (Lux)</t>
         </is>
       </c>
-      <c r="B54" t="inlineStr"/>
       <c r="C54" t="n">
         <v>25</v>
       </c>
@@ -3795,7 +3769,6 @@
           <t>EN_0364 (Lux)</t>
         </is>
       </c>
-      <c r="B55" t="inlineStr"/>
       <c r="C55" t="n">
         <v>26</v>
       </c>
@@ -3856,7 +3829,6 @@
           <t>EN_0364 (Lux)</t>
         </is>
       </c>
-      <c r="B56" t="inlineStr"/>
       <c r="C56" t="n">
         <v>27</v>
       </c>
@@ -3917,7 +3889,6 @@
           <t>EN_0364 (Lux)</t>
         </is>
       </c>
-      <c r="B57" t="inlineStr"/>
       <c r="C57" t="n">
         <v>28</v>
       </c>
@@ -3978,7 +3949,6 @@
           <t>EN_0364 (Lux)</t>
         </is>
       </c>
-      <c r="B58" t="inlineStr"/>
       <c r="C58" t="n">
         <v>29</v>
       </c>
@@ -4039,7 +4009,6 @@
           <t>EN_0364 (Lux)</t>
         </is>
       </c>
-      <c r="B59" t="inlineStr"/>
       <c r="C59" t="n">
         <v>30</v>
       </c>
@@ -4100,7 +4069,6 @@
           <t>EN_0364 (Lux)</t>
         </is>
       </c>
-      <c r="B60" t="inlineStr"/>
       <c r="C60" t="n">
         <v>31</v>
       </c>
@@ -4161,7 +4129,6 @@
           <t>EN_0364 (Lux)</t>
         </is>
       </c>
-      <c r="B61" t="inlineStr"/>
       <c r="C61" t="n">
         <v>32</v>
       </c>
@@ -4222,7 +4189,6 @@
           <t>EN_0364 (Lux)</t>
         </is>
       </c>
-      <c r="B62" t="inlineStr"/>
       <c r="C62" t="n">
         <v>33</v>
       </c>
@@ -4283,7 +4249,6 @@
           <t>EN_0364 (Lux)</t>
         </is>
       </c>
-      <c r="B63" t="inlineStr"/>
       <c r="C63" t="n">
         <v>34</v>
       </c>
@@ -4344,7 +4309,6 @@
           <t>EN_0364 (Lux)</t>
         </is>
       </c>
-      <c r="B64" t="inlineStr"/>
       <c r="C64" t="n">
         <v>35</v>
       </c>
@@ -4405,7 +4369,6 @@
           <t>EN_0364 (Lux)</t>
         </is>
       </c>
-      <c r="B65" t="inlineStr"/>
       <c r="C65" t="n">
         <v>36</v>
       </c>
@@ -4466,7 +4429,6 @@
           <t>EN_0364 (Lux)</t>
         </is>
       </c>
-      <c r="B66" t="inlineStr"/>
       <c r="C66" t="n">
         <v>37</v>
       </c>
@@ -4527,7 +4489,6 @@
           <t>EN_0364 (Lux)</t>
         </is>
       </c>
-      <c r="B67" t="inlineStr"/>
       <c r="C67" t="n">
         <v>38</v>
       </c>
@@ -4588,7 +4549,6 @@
           <t>EN_0364 (Lux)</t>
         </is>
       </c>
-      <c r="B68" t="inlineStr"/>
       <c r="C68" t="n">
         <v>39</v>
       </c>
@@ -4649,7 +4609,6 @@
           <t>EN_0364 (Lux)</t>
         </is>
       </c>
-      <c r="B69" t="inlineStr"/>
       <c r="C69" t="n">
         <v>40</v>
       </c>
@@ -4710,7 +4669,6 @@
           <t>EN_0364 (Lux)</t>
         </is>
       </c>
-      <c r="B70" t="inlineStr"/>
       <c r="C70" t="n">
         <v>41</v>
       </c>
@@ -4771,7 +4729,6 @@
           <t>EN_0364 (Lux)</t>
         </is>
       </c>
-      <c r="B71" t="inlineStr"/>
       <c r="C71" t="n">
         <v>42</v>
       </c>
@@ -4832,7 +4789,6 @@
           <t>EN_0364 (Lux)</t>
         </is>
       </c>
-      <c r="B72" t="inlineStr"/>
       <c r="C72" t="n">
         <v>43</v>
       </c>
@@ -4893,7 +4849,6 @@
           <t>EN_0364 (Lux)</t>
         </is>
       </c>
-      <c r="B73" t="inlineStr"/>
       <c r="C73" t="n">
         <v>44</v>
       </c>
@@ -4954,7 +4909,6 @@
           <t>EN_0364 (Lux)</t>
         </is>
       </c>
-      <c r="B74" t="inlineStr"/>
       <c r="C74" t="n">
         <v>45</v>
       </c>
@@ -5015,7 +4969,6 @@
           <t>EN_0364 (Lux)</t>
         </is>
       </c>
-      <c r="B75" t="inlineStr"/>
       <c r="C75" t="n">
         <v>46</v>
       </c>
@@ -5076,7 +5029,6 @@
           <t>EN_0364 (Lux)</t>
         </is>
       </c>
-      <c r="B76" t="inlineStr"/>
       <c r="C76" t="n">
         <v>47</v>
       </c>

</xml_diff>